<commit_message>
Republish Pau_2025_WC: Kayak Cross individual (Time Trials) RANK from official classification (129 cells; maintainer 2026-10-21)
</commit_message>
<xml_diff>
--- a/events/Pau_2025_WC/Pau_2025_WC_start.xlsx
+++ b/events/Pau_2025_WC/Pau_2025_WC_start.xlsx
@@ -19335,6 +19335,11 @@
       <c r="K317" t="n">
         <v>316</v>
       </c>
+      <c r="M317" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
       <c r="R317" t="inlineStr">
         <is>
           <t>LOGACHEVA Taisiia</t>
@@ -19393,6 +19398,11 @@
       <c r="K318" t="n">
         <v>317</v>
       </c>
+      <c r="M318" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
       <c r="R318" t="inlineStr">
         <is>
           <t>MILLS Waris</t>
@@ -19456,6 +19466,11 @@
       <c r="K319" t="n">
         <v>318</v>
       </c>
+      <c r="M319" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
       <c r="R319" t="inlineStr">
         <is>
           <t>LUKNAROVA Emanuela</t>
@@ -19519,6 +19534,11 @@
       <c r="K320" t="n">
         <v>319</v>
       </c>
+      <c r="M320" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
       <c r="R320" t="inlineStr">
         <is>
           <t>KRYLOVA Kseniia</t>
@@ -19582,6 +19602,11 @@
       <c r="K321" t="n">
         <v>320</v>
       </c>
+      <c r="M321" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
       <c r="R321" t="inlineStr">
         <is>
           <t>MINAZOVA Alsu</t>
@@ -19645,6 +19670,11 @@
       <c r="K322" t="n">
         <v>321</v>
       </c>
+      <c r="M322" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
       <c r="R322" t="inlineStr">
         <is>
           <t>CHEN Lin</t>
@@ -19708,6 +19738,11 @@
       <c r="K323" t="n">
         <v>322</v>
       </c>
+      <c r="M323" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
       <c r="R323" t="inlineStr">
         <is>
           <t>NESNIDALOVA Lucie</t>
@@ -19771,6 +19806,11 @@
       <c r="K324" t="n">
         <v>323</v>
       </c>
+      <c r="M324" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
       <c r="R324" t="inlineStr">
         <is>
           <t>HERZOG Andrea</t>
@@ -19834,6 +19874,11 @@
       <c r="K325" t="n">
         <v>324</v>
       </c>
+      <c r="M325" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
       <c r="R325" t="inlineStr">
         <is>
           <t>BAYN Nele</t>
@@ -19897,6 +19942,11 @@
       <c r="K326" t="n">
         <v>325</v>
       </c>
+      <c r="M326" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
       <c r="R326" t="inlineStr">
         <is>
           <t>OLSON Beatrice</t>
@@ -19960,6 +20010,11 @@
       <c r="K327" t="n">
         <v>326</v>
       </c>
+      <c r="M327" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
       <c r="R327" t="inlineStr">
         <is>
           <t>TARANTSEVA Yekaterina</t>
@@ -20023,6 +20078,11 @@
       <c r="K328" t="n">
         <v>327</v>
       </c>
+      <c r="M328" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
       <c r="R328" t="inlineStr">
         <is>
           <t>ANANYEVA Anastassiya</t>
@@ -20086,6 +20146,11 @@
       <c r="K329" t="n">
         <v>328</v>
       </c>
+      <c r="M329" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
       <c r="R329" t="inlineStr">
         <is>
           <t>PITCHER FARRELL Cleo</t>
@@ -20149,6 +20214,11 @@
       <c r="K330" t="n">
         <v>329</v>
       </c>
+      <c r="M330" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
       <c r="R330" t="inlineStr">
         <is>
           <t>SOMMERNES Iris</t>
@@ -20212,6 +20282,11 @@
       <c r="K331" t="n">
         <v>330</v>
       </c>
+      <c r="M331" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
       <c r="R331" t="inlineStr">
         <is>
           <t>MATTI Svenja</t>
@@ -20275,6 +20350,11 @@
       <c r="K332" t="n">
         <v>331</v>
       </c>
+      <c r="M332" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
       <c r="R332" t="inlineStr">
         <is>
           <t>PELLICER CHICA Laura</t>
@@ -20338,6 +20418,11 @@
       <c r="K333" t="n">
         <v>332</v>
       </c>
+      <c r="M333" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
       <c r="R333" t="inlineStr">
         <is>
           <t>WAN Shunfang</t>
@@ -20401,6 +20486,11 @@
       <c r="K334" t="n">
         <v>333</v>
       </c>
+      <c r="M334" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
       <c r="R334" t="inlineStr">
         <is>
           <t>SAMKOVA Olga</t>
@@ -20464,6 +20554,11 @@
       <c r="K335" t="n">
         <v>334</v>
       </c>
+      <c r="M335" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
       <c r="R335" t="inlineStr">
         <is>
           <t>GORA Aleksandra</t>
@@ -20527,6 +20622,11 @@
       <c r="K336" t="n">
         <v>335</v>
       </c>
+      <c r="M336" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
       <c r="R336" t="inlineStr">
         <is>
           <t>SORRIBES Laia</t>
@@ -20590,6 +20690,11 @@
       <c r="K337" t="n">
         <v>336</v>
       </c>
+      <c r="M337" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
       <c r="R337" t="inlineStr">
         <is>
           <t>WILLIAMS Courtney</t>
@@ -20653,6 +20758,11 @@
       <c r="K338" t="n">
         <v>337</v>
       </c>
+      <c r="M338" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
       <c r="R338" t="inlineStr">
         <is>
           <t>LEAVER Lois</t>
@@ -20716,6 +20826,11 @@
       <c r="K339" t="n">
         <v>338</v>
       </c>
+      <c r="M339" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
       <c r="R339" t="inlineStr">
         <is>
           <t>BALDONI Lea</t>
@@ -20779,6 +20894,11 @@
       <c r="K340" t="n">
         <v>339</v>
       </c>
+      <c r="M340" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
       <c r="R340" t="inlineStr">
         <is>
           <t>O'CALLAGHAN Georgia</t>
@@ -20842,6 +20962,11 @@
       <c r="K341" t="n">
         <v>340</v>
       </c>
+      <c r="M341" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
       <c r="R341" t="inlineStr">
         <is>
           <t>ALTMAN Marcella</t>
@@ -20905,6 +21030,11 @@
       <c r="K342" t="n">
         <v>341</v>
       </c>
+      <c r="M342" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
       <c r="R342" t="inlineStr">
         <is>
           <t>PANKOVA Zuzana</t>
@@ -20968,6 +21098,11 @@
       <c r="K343" t="n">
         <v>342</v>
       </c>
+      <c r="M343" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
       <c r="R343" t="inlineStr">
         <is>
           <t>STANOVSKA Sona</t>
@@ -21031,6 +21166,11 @@
       <c r="K344" t="n">
         <v>343</v>
       </c>
+      <c r="M344" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="R344" t="inlineStr">
         <is>
           <t>NOVAK Ajda</t>
@@ -21094,6 +21234,11 @@
       <c r="K345" t="n">
         <v>344</v>
       </c>
+      <c r="M345" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
       <c r="R345" t="inlineStr">
         <is>
           <t>SABATTINI Chiara</t>
@@ -21157,6 +21302,11 @@
       <c r="K346" t="n">
         <v>345</v>
       </c>
+      <c r="M346" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
       <c r="R346" t="inlineStr">
         <is>
           <t>HOCEVAR Eva Alina</t>
@@ -21220,6 +21370,11 @@
       <c r="K347" t="n">
         <v>346</v>
       </c>
+      <c r="M347" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
       <c r="R347" t="inlineStr">
         <is>
           <t>LAZKANO Miren</t>
@@ -21283,6 +21438,11 @@
       <c r="K348" t="n">
         <v>347</v>
       </c>
+      <c r="M348" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
       <c r="R348" t="inlineStr">
         <is>
           <t>TEUNISSEN Lena</t>
@@ -21346,6 +21506,11 @@
       <c r="K349" t="n">
         <v>348</v>
       </c>
+      <c r="M349" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
       <c r="R349" t="inlineStr">
         <is>
           <t>XIE Xueting</t>
@@ -21409,6 +21574,11 @@
       <c r="K350" t="n">
         <v>349</v>
       </c>
+      <c r="M350" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
       <c r="R350" t="inlineStr">
         <is>
           <t>US Viktoriia</t>
@@ -21472,6 +21642,11 @@
       <c r="K351" t="n">
         <v>350</v>
       </c>
+      <c r="M351" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
       <c r="R351" t="inlineStr">
         <is>
           <t>KNEBLOVA Tereza</t>
@@ -21535,6 +21710,11 @@
       <c r="K352" t="n">
         <v>351</v>
       </c>
+      <c r="M352" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
       <c r="R352" t="inlineStr">
         <is>
           <t>DORIA Monica</t>
@@ -21598,6 +21778,11 @@
       <c r="K353" t="n">
         <v>352</v>
       </c>
+      <c r="M353" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="R353" t="inlineStr">
         <is>
           <t>FOX Jessica</t>
@@ -21661,6 +21846,11 @@
       <c r="K354" t="n">
         <v>353</v>
       </c>
+      <c r="M354" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="R354" t="inlineStr">
         <is>
           <t>SETCHELL Nikita</t>
@@ -21724,6 +21914,11 @@
       <c r="K355" t="n">
         <v>354</v>
       </c>
+      <c r="M355" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
       <c r="R355" t="inlineStr">
         <is>
           <t>VUITTON Emma</t>
@@ -21787,6 +21982,11 @@
       <c r="K356" t="n">
         <v>355</v>
       </c>
+      <c r="M356" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
       <c r="R356" t="inlineStr">
         <is>
           <t>LEIBFARTH Evy</t>
@@ -21850,6 +22050,11 @@
       <c r="K357" t="n">
         <v>356</v>
       </c>
+      <c r="M357" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
       <c r="R357" t="inlineStr">
         <is>
           <t>FUNK Ricarda</t>
@@ -21913,6 +22118,11 @@
       <c r="K358" t="n">
         <v>357</v>
       </c>
+      <c r="M358" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
       <c r="R358" t="inlineStr">
         <is>
           <t>MARX Alena</t>
@@ -21976,6 +22186,11 @@
       <c r="K359" t="n">
         <v>358</v>
       </c>
+      <c r="M359" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
       <c r="R359" t="inlineStr">
         <is>
           <t>CHOURRAUT Maialen</t>
@@ -22039,6 +22254,11 @@
       <c r="K360" t="n">
         <v>359</v>
       </c>
+      <c r="M360" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
       <c r="R360" t="inlineStr">
         <is>
           <t>FOX Noemie</t>
@@ -22102,6 +22322,11 @@
       <c r="K361" t="n">
         <v>360</v>
       </c>
+      <c r="M361" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="R361" t="inlineStr">
         <is>
           <t>PRIGENT Camille</t>
@@ -22165,6 +22390,11 @@
       <c r="K362" t="n">
         <v>361</v>
       </c>
+      <c r="M362" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
       <c r="R362" t="inlineStr">
         <is>
           <t>HUG Angele</t>
@@ -22228,6 +22458,11 @@
       <c r="K363" t="n">
         <v>362</v>
       </c>
+      <c r="M363" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
       <c r="R363" t="inlineStr">
         <is>
           <t>WOODS Kimberley</t>
@@ -22291,6 +22526,11 @@
       <c r="K364" t="n">
         <v>363</v>
       </c>
+      <c r="M364" t="inlineStr">
+        <is>
+          <t>78</t>
+        </is>
+      </c>
       <c r="R364" t="inlineStr">
         <is>
           <t>ABDULLAEV Khayotbek</t>
@@ -22354,6 +22594,11 @@
       <c r="K365" t="n">
         <v>364</v>
       </c>
+      <c r="M365" t="inlineStr">
+        <is>
+          <t>77</t>
+        </is>
+      </c>
       <c r="R365" t="inlineStr">
         <is>
           <t>CHANG Fu-Hua</t>
@@ -22417,6 +22662,11 @@
       <c r="K366" t="n">
         <v>365</v>
       </c>
+      <c r="M366" t="inlineStr">
+        <is>
+          <t>75</t>
+        </is>
+      </c>
       <c r="R366" t="inlineStr">
         <is>
           <t>EIGEL Pavel</t>
@@ -22480,6 +22730,11 @@
       <c r="K367" t="n">
         <v>366</v>
       </c>
+      <c r="M367" t="inlineStr">
+        <is>
+          <t>81</t>
+        </is>
+      </c>
       <c r="R367" t="inlineStr">
         <is>
           <t>CHU Hung-Yu</t>
@@ -22543,6 +22798,11 @@
       <c r="K368" t="n">
         <v>367</v>
       </c>
+      <c r="M368" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
       <c r="R368" t="inlineStr">
         <is>
           <t>SMIRNOV Egor</t>
@@ -22606,6 +22866,11 @@
       <c r="K369" t="n">
         <v>368</v>
       </c>
+      <c r="M369" t="inlineStr">
+        <is>
+          <t>71</t>
+        </is>
+      </c>
       <c r="R369" t="inlineStr">
         <is>
           <t>AMANBAYEV Adil</t>
@@ -22669,6 +22934,11 @@
       <c r="K370" t="n">
         <v>369</v>
       </c>
+      <c r="M370" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
       <c r="R370" t="inlineStr">
         <is>
           <t>SAYDULLAEV Samandar</t>
@@ -22732,6 +23002,11 @@
       <c r="K371" t="n">
         <v>370</v>
       </c>
+      <c r="M371" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
       <c r="R371" t="inlineStr">
         <is>
           <t>GUBENKO Nikita</t>
@@ -22795,6 +23070,11 @@
       <c r="K372" t="n">
         <v>371</v>
       </c>
+      <c r="M372" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
       <c r="R372" t="inlineStr">
         <is>
           <t>KOZLOV Ivan</t>
@@ -22858,6 +23138,11 @@
       <c r="K373" t="n">
         <v>372</v>
       </c>
+      <c r="M373" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
       <c r="R373" t="inlineStr">
         <is>
           <t>NIJHAWAN Nikhil</t>
@@ -22921,6 +23206,11 @@
       <c r="K374" t="n">
         <v>373</v>
       </c>
+      <c r="M374" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
       <c r="R374" t="inlineStr">
         <is>
           <t>CHECA BARO Nil</t>
@@ -22984,6 +23274,11 @@
       <c r="K375" t="n">
         <v>374</v>
       </c>
+      <c r="M375" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
       <c r="R375" t="inlineStr">
         <is>
           <t>SNOOK George</t>
@@ -23047,6 +23342,11 @@
       <c r="K376" t="n">
         <v>375</v>
       </c>
+      <c r="M376" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
       <c r="R376" t="inlineStr">
         <is>
           <t>MUTO Yusuke</t>
@@ -23110,6 +23410,11 @@
       <c r="K377" t="n">
         <v>376</v>
       </c>
+      <c r="M377" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
       <c r="R377" t="inlineStr">
         <is>
           <t>MARIEN Martin</t>
@@ -23173,6 +23478,11 @@
       <c r="K378" t="n">
         <v>377</v>
       </c>
+      <c r="M378" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
       <c r="R378" t="inlineStr">
         <is>
           <t>STEINBRENNER Max</t>
@@ -23236,6 +23546,11 @@
       <c r="K379" t="n">
         <v>378</v>
       </c>
+      <c r="M379" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
       <c r="R379" t="inlineStr">
         <is>
           <t>MING Xingzhou</t>
@@ -23299,6 +23614,11 @@
       <c r="K380" t="n">
         <v>379</v>
       </c>
+      <c r="M380" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
       <c r="R380" t="inlineStr">
         <is>
           <t>LOCNIKAR Jan</t>
@@ -23362,6 +23682,11 @@
       <c r="K381" t="n">
         <v>380</v>
       </c>
+      <c r="M381" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
       <c r="R381" t="inlineStr">
         <is>
           <t>MAPELLI Guilherme</t>
@@ -23425,6 +23750,11 @@
       <c r="K382" t="n">
         <v>381</v>
       </c>
+      <c r="M382" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
       <c r="R382" t="inlineStr">
         <is>
           <t>ZHANG Hejie</t>
@@ -23488,6 +23818,11 @@
       <c r="K383" t="n">
         <v>382</v>
       </c>
+      <c r="M383" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
       <c r="R383" t="inlineStr">
         <is>
           <t>RUDORFER Martin</t>
@@ -23551,6 +23886,11 @@
       <c r="K384" t="n">
         <v>383</v>
       </c>
+      <c r="M384" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
       <c r="R384" t="inlineStr">
         <is>
           <t>KOROBOV Alexandr</t>
@@ -23614,6 +23954,11 @@
       <c r="K385" t="n">
         <v>384</v>
       </c>
+      <c r="M385" t="inlineStr">
+        <is>
+          <t>79</t>
+        </is>
+      </c>
       <c r="R385" t="inlineStr">
         <is>
           <t>GONSENICA Adam</t>
@@ -23677,6 +24022,11 @@
       <c r="K386" t="n">
         <v>385</v>
       </c>
+      <c r="M386" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
       <c r="R386" t="inlineStr">
         <is>
           <t>TANAKA Yuuki</t>
@@ -23740,6 +24090,11 @@
       <c r="K387" t="n">
         <v>386</v>
       </c>
+      <c r="M387" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
       <c r="R387" t="inlineStr">
         <is>
           <t>CANO MOLE Luca</t>
@@ -23803,6 +24158,11 @@
       <c r="K388" t="n">
         <v>387</v>
       </c>
+      <c r="M388" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
       <c r="R388" t="inlineStr">
         <is>
           <t>EICHFELD Casey</t>
@@ -23866,6 +24226,11 @@
       <c r="K389" t="n">
         <v>388</v>
       </c>
+      <c r="M389" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
       <c r="R389" t="inlineStr">
         <is>
           <t>GRIGAR Jakub</t>
@@ -23929,6 +24294,11 @@
       <c r="K390" t="n">
         <v>389</v>
       </c>
+      <c r="M390" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
       <c r="R390" t="inlineStr">
         <is>
           <t>ROZENTALS Klass Francisks</t>
@@ -23992,6 +24362,11 @@
       <c r="K391" t="n">
         <v>390</v>
       </c>
+      <c r="M391" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
       <c r="R391" t="inlineStr">
         <is>
           <t>HAYLETT Ben</t>
@@ -24055,6 +24430,11 @@
       <c r="K392" t="n">
         <v>391</v>
       </c>
+      <c r="M392" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
       <c r="R392" t="inlineStr">
         <is>
           <t>BARAT Andy</t>
@@ -24118,6 +24498,11 @@
       <c r="K393" t="n">
         <v>392</v>
       </c>
+      <c r="M393" t="inlineStr">
+        <is>
+          <t>73</t>
+        </is>
+      </c>
       <c r="R393" t="inlineStr">
         <is>
           <t>SARAMANDIF Terence</t>
@@ -24181,6 +24566,11 @@
       <c r="K394" t="n">
         <v>393</v>
       </c>
+      <c r="M394" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
+      </c>
       <c r="R394" t="inlineStr">
         <is>
           <t>JACOB Lucas</t>
@@ -24244,6 +24634,11 @@
       <c r="K395" t="n">
         <v>394</v>
       </c>
+      <c r="M395" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
       <c r="R395" t="inlineStr">
         <is>
           <t>UKALOVIC Thomas</t>
@@ -24307,6 +24702,11 @@
       <c r="K396" t="n">
         <v>395</v>
       </c>
+      <c r="M396" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
       <c r="R396" t="inlineStr">
         <is>
           <t>HUANG Liman</t>
@@ -24370,6 +24770,11 @@
       <c r="K397" t="n">
         <v>396</v>
       </c>
+      <c r="M397" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
       <c r="R397" t="inlineStr">
         <is>
           <t>CUNHA Joao</t>
@@ -24433,6 +24838,11 @@
       <c r="K398" t="n">
         <v>397</v>
       </c>
+      <c r="M398" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
       <c r="R398" t="inlineStr">
         <is>
           <t>ZIELONKA Mark</t>
@@ -24496,6 +24906,11 @@
       <c r="K399" t="n">
         <v>398</v>
       </c>
+      <c r="M399" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
       <c r="R399" t="inlineStr">
         <is>
           <t>SOVKO Serhii</t>
@@ -24559,6 +24974,11 @@
       <c r="K400" t="n">
         <v>399</v>
       </c>
+      <c r="M400" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
       <c r="R400" t="inlineStr">
         <is>
           <t>BOYD Trevor</t>
@@ -24622,6 +25042,11 @@
       <c r="K401" t="n">
         <v>400</v>
       </c>
+      <c r="M401" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
       <c r="R401" t="inlineStr">
         <is>
           <t>JEGOU Liam</t>
@@ -24685,6 +25110,11 @@
       <c r="K402" t="n">
         <v>401</v>
       </c>
+      <c r="M402" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
       <c r="R402" t="inlineStr">
         <is>
           <t>PUCHNER Oliver</t>
@@ -24748,6 +25178,11 @@
       <c r="K403" t="n">
         <v>402</v>
       </c>
+      <c r="M403" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
       <c r="R403" t="inlineStr">
         <is>
           <t>TRIPANO Manuel</t>
@@ -24811,6 +25246,11 @@
       <c r="K404" t="n">
         <v>403</v>
       </c>
+      <c r="M404" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
       <c r="R404" t="inlineStr">
         <is>
           <t>FRIEDENSON Kaelin</t>
@@ -24874,6 +25314,11 @@
       <c r="K405" t="n">
         <v>404</v>
       </c>
+      <c r="M405" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
       <c r="R405" t="inlineStr">
         <is>
           <t>BRZEZINSKI Jakub</t>
@@ -24937,6 +25382,11 @@
       <c r="K406" t="n">
         <v>405</v>
       </c>
+      <c r="M406" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
       <c r="R406" t="inlineStr">
         <is>
           <t>ECHANIZ Pau</t>
@@ -25000,6 +25450,11 @@
       <c r="K407" t="n">
         <v>406</v>
       </c>
+      <c r="M407" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
       <c r="R407" t="inlineStr">
         <is>
           <t>FERRAZZI Xabier</t>
@@ -25063,6 +25518,11 @@
       <c r="K408" t="n">
         <v>407</v>
       </c>
+      <c r="M408" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
       <c r="R408" t="inlineStr">
         <is>
           <t>AUBERTIN Maxime</t>
@@ -25126,6 +25586,11 @@
       <c r="K409" t="n">
         <v>408</v>
       </c>
+      <c r="M409" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="R409" t="inlineStr">
         <is>
           <t>NOVAK Matyas</t>
@@ -25189,6 +25654,11 @@
       <c r="K410" t="n">
         <v>409</v>
       </c>
+      <c r="M410" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
       <c r="R410" t="inlineStr">
         <is>
           <t>PASIUT Michal</t>
@@ -25252,6 +25722,11 @@
       <c r="K411" t="n">
         <v>410</v>
       </c>
+      <c r="M411" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
       <c r="R411" t="inlineStr">
         <is>
           <t>MARTINEZ Jesus</t>
@@ -25315,6 +25790,11 @@
       <c r="K412" t="n">
         <v>411</v>
       </c>
+      <c r="M412" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
       <c r="R412" t="inlineStr">
         <is>
           <t>IVCHENKO Artem</t>
@@ -25378,6 +25858,11 @@
       <c r="K413" t="n">
         <v>412</v>
       </c>
+      <c r="M413" t="inlineStr">
+        <is>
+          <t>59</t>
+        </is>
+      </c>
       <c r="R413" t="inlineStr">
         <is>
           <t>PEREZ RINCON Alexis</t>
@@ -25441,6 +25926,11 @@
       <c r="K414" t="n">
         <v>413</v>
       </c>
+      <c r="M414" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
       <c r="R414" t="inlineStr">
         <is>
           <t>SAVLI Jakob</t>
@@ -25504,6 +25994,11 @@
       <c r="K415" t="n">
         <v>414</v>
       </c>
+      <c r="M415" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
       <c r="R415" t="inlineStr">
         <is>
           <t>ALVARENGA Frederico</t>
@@ -25567,6 +26062,11 @@
       <c r="K416" t="n">
         <v>415</v>
       </c>
+      <c r="M416" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
       <c r="R416" t="inlineStr">
         <is>
           <t>MCCREERY Alistair</t>
@@ -25630,6 +26130,11 @@
       <c r="K417" t="n">
         <v>416</v>
       </c>
+      <c r="M417" t="inlineStr">
+        <is>
+          <t>74</t>
+        </is>
+      </c>
       <c r="R417" t="inlineStr">
         <is>
           <t>HALCIN Martin</t>
@@ -25693,6 +26198,11 @@
       <c r="K418" t="n">
         <v>417</v>
       </c>
+      <c r="M418" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
       <c r="R418" t="inlineStr">
         <is>
           <t>POPE Benjamin</t>
@@ -25756,6 +26266,11 @@
       <c r="K419" t="n">
         <v>418</v>
       </c>
+      <c r="M419" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
       <c r="R419" t="inlineStr">
         <is>
           <t>ROELLER Tillmann</t>
@@ -25819,6 +26334,11 @@
       <c r="K420" t="n">
         <v>419</v>
       </c>
+      <c r="M420" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
       <c r="R420" t="inlineStr">
         <is>
           <t>OHRSTROM Isak</t>
@@ -25882,6 +26402,11 @@
       <c r="K421" t="n">
         <v>420</v>
       </c>
+      <c r="M421" t="inlineStr">
+        <is>
+          <t>82</t>
+        </is>
+      </c>
       <c r="R421" t="inlineStr">
         <is>
           <t>DESNOS Mathieu</t>
@@ -25945,6 +26470,11 @@
       <c r="K422" t="n">
         <v>421</v>
       </c>
+      <c r="M422" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
       <c r="R422" t="inlineStr">
         <is>
           <t>BALDONI Alex</t>
@@ -26008,6 +26538,11 @@
       <c r="K423" t="n">
         <v>422</v>
       </c>
+      <c r="M423" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
       <c r="R423" t="inlineStr">
         <is>
           <t>DE COSTER Gabriel</t>
@@ -26071,6 +26606,11 @@
       <c r="K424" t="n">
         <v>423</v>
       </c>
+      <c r="M424" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
       <c r="R424" t="inlineStr">
         <is>
           <t>HENGST Stefan</t>
@@ -26134,6 +26674,11 @@
       <c r="K425" t="n">
         <v>424</v>
       </c>
+      <c r="M425" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="R425" t="inlineStr">
         <is>
           <t>KREJCI Jakub</t>
@@ -26197,6 +26742,11 @@
       <c r="K426" t="n">
         <v>425</v>
       </c>
+      <c r="M426" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
       <c r="R426" t="inlineStr">
         <is>
           <t>HOCEVAR Ziga Lin</t>
@@ -26260,6 +26810,11 @@
       <c r="K427" t="n">
         <v>426</v>
       </c>
+      <c r="M427" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
       <c r="R427" t="inlineStr">
         <is>
           <t>DELFOUR Lucien</t>
@@ -26323,6 +26878,11 @@
       <c r="K428" t="n">
         <v>427</v>
       </c>
+      <c r="M428" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
       <c r="R428" t="inlineStr">
         <is>
           <t>OSCHMAUTZ Felix</t>
@@ -26386,6 +26946,11 @@
       <c r="K429" t="n">
         <v>428</v>
       </c>
+      <c r="M429" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
       <c r="R429" t="inlineStr">
         <is>
           <t>CASTRYCK Titouan</t>
@@ -26449,6 +27014,11 @@
       <c r="K430" t="n">
         <v>429</v>
       </c>
+      <c r="M430" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="R430" t="inlineStr">
         <is>
           <t>LEAVER Sam</t>
@@ -26512,6 +27082,11 @@
       <c r="K431" t="n">
         <v>430</v>
       </c>
+      <c r="M431" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
       <c r="R431" t="inlineStr">
         <is>
           <t>ANDERSON Timothy</t>
@@ -26575,6 +27150,11 @@
       <c r="K432" t="n">
         <v>431</v>
       </c>
+      <c r="M432" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
       <c r="R432" t="inlineStr">
         <is>
           <t>DICKSON Jonny</t>
@@ -26638,6 +27218,11 @@
       <c r="K433" t="n">
         <v>432</v>
       </c>
+      <c r="M433" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
       <c r="R433" t="inlineStr">
         <is>
           <t>ECHEVERRIA OLGUIN Andraz</t>
@@ -26701,6 +27286,11 @@
       <c r="K434" t="n">
         <v>433</v>
       </c>
+      <c r="M434" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
       <c r="R434" t="inlineStr">
         <is>
           <t>ROHRER Jan</t>
@@ -26764,6 +27354,11 @@
       <c r="K435" t="n">
         <v>434</v>
       </c>
+      <c r="M435" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
       <c r="R435" t="inlineStr">
         <is>
           <t>MADORE Mathurin</t>
@@ -26827,6 +27422,11 @@
       <c r="K436" t="n">
         <v>435</v>
       </c>
+      <c r="M436" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
       <c r="R436" t="inlineStr">
         <is>
           <t>GONCALVES Pedro</t>
@@ -26890,6 +27490,11 @@
       <c r="K437" t="n">
         <v>436</v>
       </c>
+      <c r="M437" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
       <c r="R437" t="inlineStr">
         <is>
           <t>OCHOA Manuel</t>
@@ -26953,6 +27558,11 @@
       <c r="K438" t="n">
         <v>437</v>
       </c>
+      <c r="M438" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
       <c r="R438" t="inlineStr">
         <is>
           <t>HEGGE Noah</t>
@@ -27016,6 +27626,11 @@
       <c r="K439" t="n">
         <v>438</v>
       </c>
+      <c r="M439" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
       <c r="R439" t="inlineStr">
         <is>
           <t>DE GENNARO Giovanni</t>
@@ -27079,6 +27694,11 @@
       <c r="K440" t="n">
         <v>439</v>
       </c>
+      <c r="M440" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="R440" t="inlineStr">
         <is>
           <t>POLACZYK Mateusz</t>
@@ -27142,6 +27762,11 @@
       <c r="K441" t="n">
         <v>440</v>
       </c>
+      <c r="M441" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
       <c r="R441" t="inlineStr">
         <is>
           <t>LLORENTE David</t>
@@ -27205,6 +27830,11 @@
       <c r="K442" t="n">
         <v>441</v>
       </c>
+      <c r="M442" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
       <c r="R442" t="inlineStr">
         <is>
           <t>RENIA Benjamin</t>
@@ -27268,6 +27898,11 @@
       <c r="K443" t="n">
         <v>442</v>
       </c>
+      <c r="M443" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
       <c r="R443" t="inlineStr">
         <is>
           <t>MARX Dimitri</t>
@@ -27331,6 +27966,11 @@
       <c r="K444" t="n">
         <v>443</v>
       </c>
+      <c r="M444" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
       <c r="R444" t="inlineStr">
         <is>
           <t>DOUGOUD Martin</t>
@@ -27393,6 +28033,11 @@
       </c>
       <c r="K445" t="n">
         <v>444</v>
+      </c>
+      <c r="M445" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
       </c>
       <c r="R445" t="inlineStr">
         <is>

</xml_diff>